<commit_message>
Add optional mood emoji and caption to Mission; Pose 1 wording
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01437rANtd5MAYdKDkxZsNAs
</commit_message>
<xml_diff>
--- a/final-plan/Final-Plan-Pose-List.xlsx
+++ b/final-plan/Final-Plan-Pose-List.xlsx
@@ -467,7 +467,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Lie flat on your back and take it looking up</t>
+          <t>Take a picture lying down on your back</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -615,7 +615,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -631,7 +630,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -647,7 +645,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -663,7 +660,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -679,7 +675,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -695,7 +690,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -711,7 +705,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -727,7 +720,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -743,7 +735,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -759,7 +750,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -775,7 +765,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -791,7 +780,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -807,7 +795,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -823,7 +810,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -839,7 +825,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -855,7 +840,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -871,7 +855,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -887,7 +870,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -903,7 +885,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -919,7 +900,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -935,7 +915,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -951,7 +930,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -967,7 +945,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -983,7 +960,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -999,7 +975,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1015,7 +990,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1031,7 +1005,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1047,7 +1020,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1063,7 +1035,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1079,7 +1050,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -1095,7 +1065,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -1111,7 +1080,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -1127,7 +1095,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -1143,7 +1110,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -1159,7 +1125,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -1175,7 +1140,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -1191,7 +1155,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -1207,7 +1170,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -1223,7 +1185,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -1239,7 +1200,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -1255,7 +1215,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -1271,7 +1230,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -1287,7 +1245,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -1303,7 +1260,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -1319,7 +1275,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -1335,7 +1290,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -1351,7 +1305,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -1367,7 +1320,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -1383,7 +1335,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -1399,7 +1350,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -1415,7 +1365,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -1431,7 +1380,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -1447,7 +1395,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -1463,7 +1410,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -1479,7 +1425,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -1495,7 +1440,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -1511,7 +1455,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -1527,7 +1470,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -1543,7 +1485,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -1559,7 +1500,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -1575,7 +1515,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -1591,7 +1530,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -1607,7 +1545,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -1623,7 +1560,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -1639,7 +1575,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -1655,7 +1590,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -1671,7 +1605,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -1687,7 +1620,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -1703,7 +1635,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -1719,7 +1650,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -1735,7 +1665,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -1751,7 +1680,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -1767,7 +1695,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -1783,7 +1710,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -1799,7 +1725,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -1815,7 +1740,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -1831,7 +1755,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -1847,7 +1770,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -1863,7 +1785,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -1879,7 +1800,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -1895,7 +1815,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -1911,7 +1830,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -1927,7 +1845,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -1943,7 +1860,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -1959,7 +1875,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -1975,7 +1890,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -1991,7 +1905,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -2007,7 +1920,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -2023,7 +1935,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -2039,7 +1950,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -2055,7 +1965,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -2071,7 +1980,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -2087,7 +1995,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -2103,7 +2010,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -2119,7 +2025,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -2135,7 +2040,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -2151,7 +2055,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -2167,7 +2070,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -2183,7 +2085,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -2199,7 +2100,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -2215,7 +2115,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -2231,7 +2130,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -2247,7 +2145,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -2263,7 +2160,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -2279,7 +2175,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -2295,7 +2190,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -2311,7 +2205,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -2327,7 +2220,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -2343,7 +2235,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -2359,7 +2250,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -2375,7 +2265,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -2391,7 +2280,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="n">
@@ -2407,7 +2295,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -2423,7 +2310,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -2439,7 +2325,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -2455,7 +2340,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -2471,7 +2355,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -2487,7 +2370,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="n">
@@ -2503,7 +2385,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="n">
@@ -2519,7 +2400,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="n">
@@ -2535,7 +2415,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="n">
@@ -2551,7 +2430,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -2567,7 +2445,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -2583,7 +2460,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -2599,7 +2475,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -2615,7 +2490,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="n">
@@ -2631,7 +2505,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -2647,7 +2520,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="n">
@@ -2663,7 +2535,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="n">
@@ -2679,7 +2550,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -2695,7 +2565,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -2711,7 +2580,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -2727,7 +2595,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -2743,7 +2610,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="n">
@@ -2759,7 +2625,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -2775,7 +2640,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="n">
@@ -2791,7 +2655,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="n">
@@ -2807,7 +2670,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="n">
@@ -2823,7 +2685,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="n">
@@ -2839,7 +2700,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="n">
@@ -2855,7 +2715,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="n">
@@ -2871,7 +2730,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="n">
@@ -2887,7 +2745,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="n">
@@ -2903,7 +2760,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="n">
@@ -2919,7 +2775,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="n">
@@ -2935,7 +2790,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="n">
@@ -2951,7 +2805,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="n">
@@ -2967,7 +2820,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="n">
@@ -2983,7 +2835,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="n">
@@ -2999,7 +2850,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="n">
@@ -3015,7 +2865,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="n">
@@ -3031,7 +2880,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="n">
@@ -3047,7 +2895,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="n">
@@ -3063,7 +2910,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="n">
@@ -3079,7 +2925,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="n">
@@ -3095,7 +2940,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="n">
@@ -3111,7 +2955,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="n">
@@ -3127,7 +2970,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="n">
@@ -3143,7 +2985,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="n">
@@ -3159,7 +3000,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="n">
@@ -3175,7 +3015,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="n">
@@ -3191,7 +3030,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="n">
@@ -3207,7 +3045,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="n">
@@ -3223,7 +3060,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="n">
@@ -3239,7 +3075,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="n">
@@ -3255,7 +3090,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="n">
@@ -3271,7 +3105,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="n">
@@ -3287,7 +3120,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="n">
@@ -3303,7 +3135,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="n">
@@ -3319,7 +3150,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="n">
@@ -3335,7 +3165,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="n">
@@ -3351,7 +3180,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="n">
@@ -3367,7 +3195,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="n">
@@ -3383,7 +3210,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="n">
@@ -3399,7 +3225,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="n">
@@ -3415,7 +3240,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="n">
@@ -3431,7 +3255,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="n">
@@ -3447,7 +3270,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" t="n">
@@ -3463,7 +3285,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="n">
@@ -3479,7 +3300,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" t="n">
@@ -3495,7 +3315,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="n">
@@ -3511,7 +3330,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="n">
@@ -3527,7 +3345,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="n">
@@ -3543,7 +3360,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="n">
@@ -3559,7 +3375,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="n">
@@ -3575,7 +3390,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="n">
@@ -3591,7 +3405,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="n">
@@ -3607,7 +3420,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" t="n">
@@ -3623,7 +3435,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="n">
@@ -3639,7 +3450,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D198" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" t="n">
@@ -3655,7 +3465,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="n">
@@ -3671,7 +3480,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" t="n">
@@ -3687,7 +3495,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="n">
@@ -3703,7 +3510,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D202" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" t="n">
@@ -3719,7 +3525,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D203" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" t="n">
@@ -3735,7 +3540,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D204" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" t="n">
@@ -3751,7 +3555,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" t="n">
@@ -3767,7 +3570,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D206" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" t="n">
@@ -3783,7 +3585,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D207" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" t="n">
@@ -3799,7 +3600,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D208" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" t="n">
@@ -3815,7 +3615,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D209" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" t="n">
@@ -3831,7 +3630,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D210" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" t="n">
@@ -3847,7 +3645,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D211" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" t="n">
@@ -3863,7 +3660,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D212" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" t="n">
@@ -3879,7 +3675,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D213" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" t="n">
@@ -3895,7 +3690,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D214" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" t="n">
@@ -3911,7 +3705,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D215" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" t="n">
@@ -3927,7 +3720,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D216" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" t="n">
@@ -3943,7 +3735,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D217" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" t="n">
@@ -3959,7 +3750,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D218" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" t="n">
@@ -3975,7 +3765,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D219" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" t="n">
@@ -3991,7 +3780,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D220" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" t="n">
@@ -4007,7 +3795,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D221" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" t="n">
@@ -4023,7 +3810,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D222" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" t="n">
@@ -4039,7 +3825,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D223" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" t="n">
@@ -4055,7 +3840,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D224" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" t="n">
@@ -4071,7 +3855,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D225" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" t="n">
@@ -4087,7 +3870,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D226" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" t="n">
@@ -4103,7 +3885,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D227" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" t="n">
@@ -4119,7 +3900,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D228" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" t="n">
@@ -4135,7 +3915,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" t="n">
@@ -4151,7 +3930,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D230" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" t="n">
@@ -4167,7 +3945,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D231" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" t="n">
@@ -4183,7 +3960,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D232" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" t="n">
@@ -4199,7 +3975,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D233" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" t="n">
@@ -4215,7 +3990,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D234" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" t="n">
@@ -4231,7 +4005,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D235" t="inlineStr"/>
     </row>
     <row r="236">
       <c r="A236" t="n">
@@ -4247,7 +4020,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D236" t="inlineStr"/>
     </row>
     <row r="237">
       <c r="A237" t="n">
@@ -4263,7 +4035,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D237" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" t="n">
@@ -4279,7 +4050,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D238" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" t="n">
@@ -4295,7 +4065,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D239" t="inlineStr"/>
     </row>
     <row r="240">
       <c r="A240" t="n">
@@ -4311,7 +4080,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D240" t="inlineStr"/>
     </row>
     <row r="241">
       <c r="A241" t="n">
@@ -4327,7 +4095,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D241" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" t="n">
@@ -4343,7 +4110,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D242" t="inlineStr"/>
     </row>
     <row r="243">
       <c r="A243" t="n">
@@ -4359,7 +4125,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D243" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" t="n">
@@ -4375,7 +4140,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D244" t="inlineStr"/>
     </row>
     <row r="245">
       <c r="A245" t="n">
@@ -4391,7 +4155,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D245" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" t="n">
@@ -4407,7 +4170,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D246" t="inlineStr"/>
     </row>
     <row r="247">
       <c r="A247" t="n">
@@ -4423,7 +4185,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D247" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" t="n">
@@ -4439,7 +4200,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D248" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" t="n">
@@ -4455,7 +4215,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D249" t="inlineStr"/>
     </row>
     <row r="250">
       <c r="A250" t="n">
@@ -4471,7 +4230,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D250" t="inlineStr"/>
     </row>
     <row r="251">
       <c r="A251" t="n">
@@ -4487,7 +4245,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D251" t="inlineStr"/>
     </row>
     <row r="252">
       <c r="A252" t="n">
@@ -4503,7 +4260,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D252" t="inlineStr"/>
     </row>
     <row r="253">
       <c r="A253" t="n">
@@ -4519,7 +4275,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D253" t="inlineStr"/>
     </row>
     <row r="254">
       <c r="A254" t="n">
@@ -4535,7 +4290,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D254" t="inlineStr"/>
     </row>
     <row r="255">
       <c r="A255" t="n">
@@ -4551,7 +4305,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D255" t="inlineStr"/>
     </row>
     <row r="256">
       <c r="A256" t="n">
@@ -4567,7 +4320,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D256" t="inlineStr"/>
     </row>
     <row r="257">
       <c r="A257" t="n">
@@ -4583,7 +4335,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D257" t="inlineStr"/>
     </row>
     <row r="258">
       <c r="A258" t="n">
@@ -4599,7 +4350,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D258" t="inlineStr"/>
     </row>
     <row r="259">
       <c r="A259" t="n">
@@ -4615,7 +4365,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D259" t="inlineStr"/>
     </row>
     <row r="260">
       <c r="A260" t="n">
@@ -4631,7 +4380,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D260" t="inlineStr"/>
     </row>
     <row r="261">
       <c r="A261" t="n">
@@ -4647,7 +4395,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D261" t="inlineStr"/>
     </row>
     <row r="262">
       <c r="A262" t="n">
@@ -4663,7 +4410,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D262" t="inlineStr"/>
     </row>
     <row r="263">
       <c r="A263" t="n">
@@ -4679,7 +4425,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D263" t="inlineStr"/>
     </row>
     <row r="264">
       <c r="A264" t="n">
@@ -4695,7 +4440,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D264" t="inlineStr"/>
     </row>
     <row r="265">
       <c r="A265" t="n">
@@ -4711,7 +4455,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D265" t="inlineStr"/>
     </row>
     <row r="266">
       <c r="A266" t="n">
@@ -4727,7 +4470,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D266" t="inlineStr"/>
     </row>
     <row r="267">
       <c r="A267" t="n">
@@ -4743,7 +4485,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D267" t="inlineStr"/>
     </row>
     <row r="268">
       <c r="A268" t="n">
@@ -4759,7 +4500,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D268" t="inlineStr"/>
     </row>
     <row r="269">
       <c r="A269" t="n">
@@ -4775,7 +4515,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D269" t="inlineStr"/>
     </row>
     <row r="270">
       <c r="A270" t="n">
@@ -4791,7 +4530,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D270" t="inlineStr"/>
     </row>
     <row r="271">
       <c r="A271" t="n">
@@ -4807,7 +4545,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D271" t="inlineStr"/>
     </row>
     <row r="272">
       <c r="A272" t="n">
@@ -4823,7 +4560,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D272" t="inlineStr"/>
     </row>
     <row r="273">
       <c r="A273" t="n">
@@ -4839,7 +4575,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D273" t="inlineStr"/>
     </row>
     <row r="274">
       <c r="A274" t="n">
@@ -4855,7 +4590,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D274" t="inlineStr"/>
     </row>
     <row r="275">
       <c r="A275" t="n">
@@ -4871,7 +4605,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D275" t="inlineStr"/>
     </row>
     <row r="276">
       <c r="A276" t="n">
@@ -4887,7 +4620,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D276" t="inlineStr"/>
     </row>
     <row r="277">
       <c r="A277" t="n">
@@ -4903,7 +4635,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D277" t="inlineStr"/>
     </row>
     <row r="278">
       <c r="A278" t="n">
@@ -4919,7 +4650,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D278" t="inlineStr"/>
     </row>
     <row r="279">
       <c r="A279" t="n">
@@ -4935,7 +4665,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D279" t="inlineStr"/>
     </row>
     <row r="280">
       <c r="A280" t="n">
@@ -4951,7 +4680,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D280" t="inlineStr"/>
     </row>
     <row r="281">
       <c r="A281" t="n">
@@ -4967,7 +4695,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D281" t="inlineStr"/>
     </row>
     <row r="282">
       <c r="A282" t="n">
@@ -4983,7 +4710,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D282" t="inlineStr"/>
     </row>
     <row r="283">
       <c r="A283" t="n">
@@ -4999,7 +4725,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D283" t="inlineStr"/>
     </row>
     <row r="284">
       <c r="A284" t="n">
@@ -5015,7 +4740,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D284" t="inlineStr"/>
     </row>
     <row r="285">
       <c r="A285" t="n">
@@ -5031,7 +4755,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D285" t="inlineStr"/>
     </row>
     <row r="286">
       <c r="A286" t="n">
@@ -5047,7 +4770,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D286" t="inlineStr"/>
     </row>
     <row r="287">
       <c r="A287" t="n">
@@ -5063,7 +4785,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D287" t="inlineStr"/>
     </row>
     <row r="288">
       <c r="A288" t="n">
@@ -5079,7 +4800,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D288" t="inlineStr"/>
     </row>
     <row r="289">
       <c r="A289" t="n">
@@ -5095,7 +4815,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D289" t="inlineStr"/>
     </row>
     <row r="290">
       <c r="A290" t="n">
@@ -5111,7 +4830,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D290" t="inlineStr"/>
     </row>
     <row r="291">
       <c r="A291" t="n">
@@ -5127,7 +4845,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D291" t="inlineStr"/>
     </row>
     <row r="292">
       <c r="A292" t="n">
@@ -5143,7 +4860,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D292" t="inlineStr"/>
     </row>
     <row r="293">
       <c r="A293" t="n">
@@ -5159,7 +4875,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D293" t="inlineStr"/>
     </row>
     <row r="294">
       <c r="A294" t="n">
@@ -5175,7 +4890,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D294" t="inlineStr"/>
     </row>
     <row r="295">
       <c r="A295" t="n">
@@ -5191,7 +4905,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D295" t="inlineStr"/>
     </row>
     <row r="296">
       <c r="A296" t="n">
@@ -5207,7 +4920,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D296" t="inlineStr"/>
     </row>
     <row r="297">
       <c r="A297" t="n">
@@ -5223,7 +4935,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D297" t="inlineStr"/>
     </row>
     <row r="298">
       <c r="A298" t="n">
@@ -5239,7 +4950,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D298" t="inlineStr"/>
     </row>
     <row r="299">
       <c r="A299" t="n">
@@ -5255,7 +4965,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D299" t="inlineStr"/>
     </row>
     <row r="300">
       <c r="A300" t="n">
@@ -5271,7 +4980,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D300" t="inlineStr"/>
     </row>
     <row r="301">
       <c r="A301" t="n">
@@ -5287,7 +4995,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D301" t="inlineStr"/>
     </row>
     <row r="302">
       <c r="A302" t="n">
@@ -5303,7 +5010,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D302" t="inlineStr"/>
     </row>
     <row r="303">
       <c r="A303" t="n">
@@ -5319,7 +5025,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D303" t="inlineStr"/>
     </row>
     <row r="304">
       <c r="A304" t="n">
@@ -5335,7 +5040,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D304" t="inlineStr"/>
     </row>
     <row r="305">
       <c r="A305" t="n">
@@ -5351,7 +5055,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D305" t="inlineStr"/>
     </row>
     <row r="306">
       <c r="A306" t="n">
@@ -5367,7 +5070,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D306" t="inlineStr"/>
     </row>
     <row r="307">
       <c r="A307" t="n">
@@ -5383,7 +5085,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D307" t="inlineStr"/>
     </row>
     <row r="308">
       <c r="A308" t="n">
@@ -5399,7 +5100,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D308" t="inlineStr"/>
     </row>
     <row r="309">
       <c r="A309" t="n">
@@ -5415,7 +5115,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D309" t="inlineStr"/>
     </row>
     <row r="310">
       <c r="A310" t="n">
@@ -5431,7 +5130,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D310" t="inlineStr"/>
     </row>
     <row r="311">
       <c r="A311" t="n">
@@ -5447,7 +5145,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D311" t="inlineStr"/>
     </row>
     <row r="312">
       <c r="A312" t="n">
@@ -5463,7 +5160,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D312" t="inlineStr"/>
     </row>
     <row r="313">
       <c r="A313" t="n">
@@ -5479,7 +5175,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D313" t="inlineStr"/>
     </row>
     <row r="314">
       <c r="A314" t="n">
@@ -5495,7 +5190,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D314" t="inlineStr"/>
     </row>
     <row r="315">
       <c r="A315" t="n">
@@ -5511,7 +5205,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D315" t="inlineStr"/>
     </row>
     <row r="316">
       <c r="A316" t="n">
@@ -5527,7 +5220,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D316" t="inlineStr"/>
     </row>
     <row r="317">
       <c r="A317" t="n">
@@ -5543,7 +5235,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D317" t="inlineStr"/>
     </row>
     <row r="318">
       <c r="A318" t="n">
@@ -5559,7 +5250,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D318" t="inlineStr"/>
     </row>
     <row r="319">
       <c r="A319" t="n">
@@ -5575,7 +5265,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D319" t="inlineStr"/>
     </row>
     <row r="320">
       <c r="A320" t="n">
@@ -5591,7 +5280,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D320" t="inlineStr"/>
     </row>
     <row r="321">
       <c r="A321" t="n">
@@ -5607,7 +5295,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D321" t="inlineStr"/>
     </row>
     <row r="322">
       <c r="A322" t="n">
@@ -5623,7 +5310,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D322" t="inlineStr"/>
     </row>
     <row r="323">
       <c r="A323" t="n">
@@ -5639,7 +5325,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D323" t="inlineStr"/>
     </row>
     <row r="324">
       <c r="A324" t="n">
@@ -5655,7 +5340,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D324" t="inlineStr"/>
     </row>
     <row r="325">
       <c r="A325" t="n">
@@ -5671,7 +5355,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D325" t="inlineStr"/>
     </row>
     <row r="326">
       <c r="A326" t="n">
@@ -5687,7 +5370,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D326" t="inlineStr"/>
     </row>
     <row r="327">
       <c r="A327" t="n">
@@ -5703,7 +5385,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D327" t="inlineStr"/>
     </row>
     <row r="328">
       <c r="A328" t="n">
@@ -5719,7 +5400,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D328" t="inlineStr"/>
     </row>
     <row r="329">
       <c r="A329" t="n">
@@ -5735,7 +5415,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D329" t="inlineStr"/>
     </row>
     <row r="330">
       <c r="A330" t="n">
@@ -5751,7 +5430,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D330" t="inlineStr"/>
     </row>
     <row r="331">
       <c r="A331" t="n">
@@ -5767,7 +5445,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D331" t="inlineStr"/>
     </row>
     <row r="332">
       <c r="A332" t="n">
@@ -5783,7 +5460,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D332" t="inlineStr"/>
     </row>
     <row r="333">
       <c r="A333" t="n">
@@ -5799,7 +5475,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D333" t="inlineStr"/>
     </row>
     <row r="334">
       <c r="A334" t="n">
@@ -5815,7 +5490,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D334" t="inlineStr"/>
     </row>
     <row r="335">
       <c r="A335" t="n">
@@ -5831,7 +5505,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D335" t="inlineStr"/>
     </row>
     <row r="336">
       <c r="A336" t="n">
@@ -5847,7 +5520,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D336" t="inlineStr"/>
     </row>
     <row r="337">
       <c r="A337" t="n">
@@ -5863,7 +5535,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D337" t="inlineStr"/>
     </row>
     <row r="338">
       <c r="A338" t="n">
@@ -5879,7 +5550,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D338" t="inlineStr"/>
     </row>
     <row r="339">
       <c r="A339" t="n">
@@ -5895,7 +5565,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D339" t="inlineStr"/>
     </row>
     <row r="340">
       <c r="A340" t="n">
@@ -5911,7 +5580,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D340" t="inlineStr"/>
     </row>
     <row r="341">
       <c r="A341" t="n">
@@ -5927,7 +5595,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D341" t="inlineStr"/>
     </row>
     <row r="342">
       <c r="A342" t="n">
@@ -5943,7 +5610,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D342" t="inlineStr"/>
     </row>
     <row r="343">
       <c r="A343" t="n">
@@ -5959,7 +5625,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D343" t="inlineStr"/>
     </row>
     <row r="344">
       <c r="A344" t="n">
@@ -5975,7 +5640,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D344" t="inlineStr"/>
     </row>
     <row r="345">
       <c r="A345" t="n">
@@ -5991,7 +5655,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D345" t="inlineStr"/>
     </row>
     <row r="346">
       <c r="A346" t="n">
@@ -6007,7 +5670,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D346" t="inlineStr"/>
     </row>
     <row r="347">
       <c r="A347" t="n">
@@ -6023,7 +5685,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D347" t="inlineStr"/>
     </row>
     <row r="348">
       <c r="A348" t="n">
@@ -6039,7 +5700,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D348" t="inlineStr"/>
     </row>
     <row r="349">
       <c r="A349" t="n">
@@ -6055,7 +5715,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D349" t="inlineStr"/>
     </row>
     <row r="350">
       <c r="A350" t="n">
@@ -6071,7 +5730,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D350" t="inlineStr"/>
     </row>
     <row r="351">
       <c r="A351" t="n">
@@ -6087,7 +5745,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D351" t="inlineStr"/>
     </row>
     <row r="352">
       <c r="A352" t="n">
@@ -6103,7 +5760,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D352" t="inlineStr"/>
     </row>
     <row r="353">
       <c r="A353" t="n">
@@ -6119,7 +5775,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D353" t="inlineStr"/>
     </row>
     <row r="354">
       <c r="A354" t="n">
@@ -6135,7 +5790,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D354" t="inlineStr"/>
     </row>
     <row r="355">
       <c r="A355" t="n">
@@ -6151,7 +5805,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D355" t="inlineStr"/>
     </row>
     <row r="356">
       <c r="A356" t="n">
@@ -6167,7 +5820,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D356" t="inlineStr"/>
     </row>
     <row r="357">
       <c r="A357" t="n">
@@ -6183,7 +5835,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D357" t="inlineStr"/>
     </row>
     <row r="358">
       <c r="A358" t="n">
@@ -6199,7 +5850,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D358" t="inlineStr"/>
     </row>
     <row r="359">
       <c r="A359" t="n">
@@ -6215,7 +5865,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D359" t="inlineStr"/>
     </row>
     <row r="360">
       <c r="A360" t="n">
@@ -6231,7 +5880,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D360" t="inlineStr"/>
     </row>
     <row r="361">
       <c r="A361" t="n">
@@ -6247,7 +5895,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D361" t="inlineStr"/>
     </row>
     <row r="362">
       <c r="A362" t="n">
@@ -6263,7 +5910,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D362" t="inlineStr"/>
     </row>
     <row r="363">
       <c r="A363" t="n">
@@ -6279,7 +5925,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D363" t="inlineStr"/>
     </row>
     <row r="364">
       <c r="A364" t="n">
@@ -6295,7 +5940,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D364" t="inlineStr"/>
     </row>
     <row r="365">
       <c r="A365" t="n">
@@ -6311,7 +5955,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D365" t="inlineStr"/>
     </row>
     <row r="366">
       <c r="A366" t="n">
@@ -6327,7 +5970,6 @@
           <t>Yes, unlimited</t>
         </is>
       </c>
-      <c r="D366" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>